<commit_message>
First half hex acc
</commit_message>
<xml_diff>
--- a/data/hex_xlsx/DIGIA.HE.xlsx
+++ b/data/hex_xlsx/DIGIA.HE.xlsx
@@ -11214,7 +11214,7 @@
       <c r="R45" s="20"/>
       <c r="S45" s="20"/>
       <c r="T45" s="20"/>
-      <c r="U45" s="20"/>
+      <c r="U45" s="19"/>
       <c r="V45" s="20"/>
       <c r="W45" s="20"/>
     </row>
@@ -11264,16 +11264,37 @@
       <c r="O46" s="19">
         <v>15.8</v>
       </c>
-      <c r="P46" s="20"/>
-      <c r="Q46" s="20"/>
+      <c r="P46" s="19">
+        <f>SUM(P48:P61)</f>
+        <v>24.42</v>
+      </c>
+      <c r="Q46" s="19">
+        <f>SUM(Q61,Q57,Q53,Q52,Q51,Q49,Q48,Q47)</f>
+        <v>36.2</v>
+      </c>
       <c r="R46" s="19">
         <v>21.7</v>
       </c>
-      <c r="S46" s="20"/>
-      <c r="T46" s="20"/>
-      <c r="U46" s="20"/>
-      <c r="V46" s="20"/>
-      <c r="W46" s="20"/>
+      <c r="S46" s="19">
+        <f t="shared" ref="S46:W46" si="1">SUM(S61,S57,S53,S52,S51,S49,S48,S47)</f>
+        <v>46.12</v>
+      </c>
+      <c r="T46" s="19">
+        <f t="shared" si="1"/>
+        <v>38.64</v>
+      </c>
+      <c r="U46" s="19">
+        <f t="shared" si="1"/>
+        <v>44.92</v>
+      </c>
+      <c r="V46" s="19">
+        <f t="shared" si="1"/>
+        <v>42.79</v>
+      </c>
+      <c r="W46" s="19">
+        <f t="shared" si="1"/>
+        <v>13.98</v>
+      </c>
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">

</xml_diff>